<commit_message>
docs: switch Word showcases to English thesis format, fix diagrams and Excel
- Regenerate Word fill showcase as English thesis with proper title size (16pt) and structured sections
- Regenerate from-scratch thesis as all-English 4-chapter document
- Remove PPT section from README and display/
- Fix Excel render to show data sheet instead of empty Sheet1
- Fix diagram generator: white background, monochrome, support attributes field
- Regenerate class/sequence/usecase diagrams with light theme
</commit_message>
<xml_diff>
--- a/display/excel/campuspulse-demo.xlsx
+++ b/display/excel/campuspulse-demo.xlsx
@@ -2,7 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
     <x:sheet name="报名统计" sheetId="2" r:id="Rb4e4fc54f876435e"/>
   </x:sheets>
   <x:calcPr fullCalcOnLoad="1"/>
@@ -166,12 +165,6 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetData/>
-</x:worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData>

</xml_diff>